<commit_message>
Ajout type tribu from BDLOC POI
</commit_message>
<xml_diff>
--- a/indexes/nc_build_all/clean_cat.xlsx
+++ b/indexes/nc_build_all/clean_cat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\maximilien\adresse\magisnc-dinum-api-adresses-f752eef9c72d\magisnc-dinum-api-adresses-f752eef9c72d\indexes\nc_build_all\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BAPA\projets\DINUM\2025_API_ADRESSE\code\magis-dinum-api-adresses\indexes\nc_build_all\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEC670D4-DA2E-4E9B-A9D9-F0BA14220E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FC51CA-705B-4822-A84F-CC9C4A25699F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="18420" yWindow="2835" windowWidth="21600" windowHeight="11385" xr2:uid="{DDE60798-8F18-41CD-9232-3F88E1F48177}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DDE60798-8F18-41CD-9232-3F88E1F48177}"/>
   </bookViews>
   <sheets>
     <sheet name="clean_cat" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -38,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
-    <t>category</t>
-  </si>
-  <si>
     <t>complet_cat</t>
   </si>
   <si>
@@ -101,9 +101,6 @@
     <t>PARC</t>
   </si>
   <si>
-    <t>PARC ESPACE PUBLIC ET LOISIR</t>
-  </si>
-  <si>
     <t>SCIVILE</t>
   </si>
   <si>
@@ -132,6 +129,12 @@
   </si>
   <si>
     <t>TRANSPORT</t>
+  </si>
+  <si>
+    <t>PARC ESPACE PUBLIC</t>
+  </si>
+  <si>
+    <t>PARC ESPACE PUBLIC ET LOISIR</t>
   </si>
 </sst>
 </file>
@@ -508,146 +511,146 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debug fichier xlsx clean_cat
</commit_message>
<xml_diff>
--- a/indexes/nc_build_all/clean_cat.xlsx
+++ b/indexes/nc_build_all/clean_cat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BAPA\projets\DINUM\2025_API_ADRESSE\code\magis-dinum-api-adresses\indexes\nc_build_all\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\maximilien\adresse\magisnc-dinum-api-adresses-f752eef9c72d\magisnc-dinum-api-adresses-f752eef9c72d\indexes\nc_build_all\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FC51CA-705B-4822-A84F-CC9C4A25699F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEC670D4-DA2E-4E9B-A9D9-F0BA14220E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DDE60798-8F18-41CD-9232-3F88E1F48177}"/>
+    <workbookView minimized="1" xWindow="18420" yWindow="2835" windowWidth="21600" windowHeight="11385" xr2:uid="{DDE60798-8F18-41CD-9232-3F88E1F48177}"/>
   </bookViews>
   <sheets>
     <sheet name="clean_cat" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -41,6 +38,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
+    <t>category</t>
+  </si>
+  <si>
     <t>complet_cat</t>
   </si>
   <si>
@@ -101,6 +101,9 @@
     <t>PARC</t>
   </si>
   <si>
+    <t>PARC ESPACE PUBLIC ET LOISIR</t>
+  </si>
+  <si>
     <t>SCIVILE</t>
   </si>
   <si>
@@ -129,12 +132,6 @@
   </si>
   <si>
     <t>TRANSPORT</t>
-  </si>
-  <si>
-    <t>PARC ESPACE PUBLIC</t>
-  </si>
-  <si>
-    <t>PARC ESPACE PUBLIC ET LOISIR</t>
   </si>
 </sst>
 </file>
@@ -511,146 +508,146 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>